<commit_message>
Add GUI module, update PCB design, and improve README documentation
Signed-off-by: JiaHe_Xu <jiahexu@arizona.edu>
</commit_message>
<xml_diff>
--- a/Hardware/Heater - Cooler Peltier Brick/SMD_PCB111/SMD_PCB/BOM/BOM peltier smd .xlsx
+++ b/Hardware/Heater - Cooler Peltier Brick/SMD_PCB111/SMD_PCB/BOM/BOM peltier smd .xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohth\Downloads\Heatercooler SMD_PCB\SMD_PCB\SMD_PCB\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohth\Downloads\1Peltier SMD_PCB_V3\1Peltier SMD_PCB_V3\SMD_PCB\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A01ECF24-C018-415B-B6EE-AD0184DF6371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA87853D-9F7C-4556-830B-569B4D97F710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Impedance_Potential_BOM_values" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="124">
   <si>
     <t>Item #</t>
   </si>
@@ -231,9 +231,6 @@
     <t>PinHeader_1x06_P2.54mm_Vertical</t>
   </si>
   <si>
-    <t>L_TDK_SLF12575</t>
-  </si>
-  <si>
     <t>TO-263-5_TabPin3</t>
   </si>
   <si>
@@ -264,9 +261,6 @@
     <t>Pelt1-</t>
   </si>
   <si>
-    <t>100uH</t>
-  </si>
-  <si>
     <t>Pelt2+</t>
   </si>
   <si>
@@ -324,15 +318,6 @@
     <t>CAP CER 1uF 50V X7R 1206</t>
   </si>
   <si>
-    <t>SLF12575T-101M1R9-PF</t>
-  </si>
-  <si>
-    <t>C81470</t>
-  </si>
-  <si>
-    <t>TDK</t>
-  </si>
-  <si>
     <t>1N4148W</t>
   </si>
   <si>
@@ -397,6 +382,21 @@
   </si>
   <si>
     <t>Minos</t>
+  </si>
+  <si>
+    <t>COILMX</t>
+  </si>
+  <si>
+    <t>MBH125-101M</t>
+  </si>
+  <si>
+    <t>C2981396</t>
+  </si>
+  <si>
+    <t>100uH 2A 178mΩ Unshielded Inductor ±20% SMD,12.5x12.5mm Fixed Inductors RoHS</t>
+  </si>
+  <si>
+    <t>SMD,12.5x12.5mm</t>
   </si>
 </sst>
 </file>
@@ -1042,19 +1042,19 @@
         <v>44</v>
       </c>
       <c r="D2" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="I2" s="6" t="s">
         <v>84</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="F2" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>86</v>
       </c>
       <c r="J2" s="6" t="s">
         <v>14</v>
@@ -1077,13 +1077,13 @@
         <v>16</v>
       </c>
       <c r="E3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" t="s">
         <v>87</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="H3" t="s">
-        <v>89</v>
       </c>
       <c r="I3" s="1">
         <v>1206</v>
@@ -1106,19 +1106,19 @@
         <v>57</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="H4" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>14</v>
@@ -1138,19 +1138,19 @@
         <v>52</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="E5" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="H5" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>14</v>
@@ -1173,14 +1173,14 @@
         <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G6"/>
       <c r="H6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="I6" s="1">
         <v>1206</v>
@@ -1204,19 +1204,19 @@
         <v>52</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E7" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="H7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>14</v>
@@ -1236,19 +1236,19 @@
         <v>55</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F8" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="H8" t="s">
         <v>93</v>
       </c>
-      <c r="H8" t="s">
-        <v>95</v>
-      </c>
       <c r="I8" s="1" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="J8" s="6" t="s">
         <v>14</v>
@@ -1271,13 +1271,13 @@
         <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I9" s="1">
         <v>1206</v>
@@ -1300,17 +1300,17 @@
         <v>44</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I10" t="s">
         <v>66</v>
@@ -1337,13 +1337,13 @@
         <v>13</v>
       </c>
       <c r="E11" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I11" s="1">
         <v>1206</v>
@@ -1366,25 +1366,27 @@
         <v>57</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="E12" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="G12"/>
       <c r="H12" t="s">
-        <v>79</v>
-      </c>
-      <c r="I12" s="1"/>
+        <v>122</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>123</v>
+      </c>
       <c r="J12" s="6" t="s">
         <v>14</v>
       </c>
       <c r="K12"/>
       <c r="L12" t="s">
-        <v>68</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -1401,22 +1403,22 @@
         <v>15</v>
       </c>
       <c r="E13" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="H13" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
@@ -1434,7 +1436,7 @@
       <c r="F14" s="19"/>
       <c r="G14" s="19"/>
       <c r="H14" s="19" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I14" s="20"/>
       <c r="J14" s="21" t="s">
@@ -1445,7 +1447,7 @@
         <v>62</v>
       </c>
       <c r="M14" s="22" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -1463,7 +1465,7 @@
       <c r="F15" s="19"/>
       <c r="G15" s="19"/>
       <c r="H15" s="19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I15" s="20"/>
       <c r="J15" s="21" t="s">
@@ -1474,7 +1476,7 @@
         <v>62</v>
       </c>
       <c r="M15" s="22" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -1492,7 +1494,7 @@
       <c r="F16" s="19"/>
       <c r="G16" s="19"/>
       <c r="H16" s="19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I16" s="20"/>
       <c r="J16" s="21" t="s">
@@ -1503,7 +1505,7 @@
         <v>67</v>
       </c>
       <c r="M16" s="22" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1521,7 +1523,7 @@
       <c r="F17" s="19"/>
       <c r="G17" s="19"/>
       <c r="H17" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I17" s="20"/>
       <c r="J17" s="21" t="s">
@@ -1532,7 +1534,7 @@
         <v>19</v>
       </c>
       <c r="M17" s="22" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1550,7 +1552,7 @@
       <c r="F18" s="19"/>
       <c r="G18" s="19"/>
       <c r="H18" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I18" s="20"/>
       <c r="J18" s="21" t="s">
@@ -1561,7 +1563,7 @@
         <v>62</v>
       </c>
       <c r="M18" s="22" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -1579,7 +1581,7 @@
       <c r="F19" s="19"/>
       <c r="G19" s="19"/>
       <c r="H19" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I19" s="20"/>
       <c r="J19" s="21" t="s">
@@ -1590,7 +1592,7 @@
         <v>62</v>
       </c>
       <c r="M19" s="22" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -1608,7 +1610,7 @@
       <c r="F20" s="19"/>
       <c r="G20" s="19"/>
       <c r="H20" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I20" s="20"/>
       <c r="J20" s="21" t="s">
@@ -1619,7 +1621,7 @@
         <v>62</v>
       </c>
       <c r="M20" s="22" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -1637,7 +1639,7 @@
       <c r="F21" s="21"/>
       <c r="G21" s="21"/>
       <c r="H21" s="19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I21" s="21"/>
       <c r="J21" s="21" t="s">
@@ -1648,7 +1650,7 @@
         <v>62</v>
       </c>
       <c r="M21" s="22" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
@@ -1964,17 +1966,17 @@
     <hyperlink ref="F9" r:id="rId10" xr:uid="{15878162-F4C0-46AA-B48A-4CE3070D260C}"/>
     <hyperlink ref="F11" r:id="rId11" xr:uid="{BC063569-3F76-46A4-A9A5-91785C9F027D}"/>
     <hyperlink ref="D11" r:id="rId12" xr:uid="{B3E2B8E0-8212-4B61-A39A-03D1133CBE20}"/>
-    <hyperlink ref="F12" r:id="rId13" xr:uid="{8F3F391D-542B-4D49-9448-4B1C53A5F4E9}"/>
-    <hyperlink ref="D12" r:id="rId14" xr:uid="{462859EF-38D5-483A-B46B-442172880E89}"/>
-    <hyperlink ref="D10" r:id="rId15" xr:uid="{EE3B7EBC-F54D-43CF-8541-5B89A52B3A4F}"/>
-    <hyperlink ref="F10" r:id="rId16" xr:uid="{9754F76B-62C5-44D0-B8AD-49EFD99D6106}"/>
-    <hyperlink ref="F13" r:id="rId17" xr:uid="{1E8D4CB2-0F9E-49A2-9C47-AE6C7817D220}"/>
-    <hyperlink ref="F5" r:id="rId18" xr:uid="{20BDEBC3-1924-4CCB-8A8E-DD75C636F1BE}"/>
-    <hyperlink ref="D5" r:id="rId19" xr:uid="{CD2E35A6-F544-4B63-A636-74D77758C266}"/>
-    <hyperlink ref="F4" r:id="rId20" xr:uid="{F3943AA0-1471-4D0C-BBB5-13FA0FC276C0}"/>
-    <hyperlink ref="D4" r:id="rId21" xr:uid="{1EFEDA74-BF37-4EFE-ADF1-10A85C773490}"/>
-    <hyperlink ref="F7" r:id="rId22" xr:uid="{D1B9C0A9-C86C-4C80-89C5-7E8FB7329756}"/>
-    <hyperlink ref="D7" r:id="rId23" xr:uid="{AB09AABC-8542-4C1B-B8C5-72F1265B0E68}"/>
+    <hyperlink ref="D10" r:id="rId13" xr:uid="{EE3B7EBC-F54D-43CF-8541-5B89A52B3A4F}"/>
+    <hyperlink ref="F10" r:id="rId14" xr:uid="{9754F76B-62C5-44D0-B8AD-49EFD99D6106}"/>
+    <hyperlink ref="F13" r:id="rId15" xr:uid="{1E8D4CB2-0F9E-49A2-9C47-AE6C7817D220}"/>
+    <hyperlink ref="F5" r:id="rId16" xr:uid="{20BDEBC3-1924-4CCB-8A8E-DD75C636F1BE}"/>
+    <hyperlink ref="D5" r:id="rId17" xr:uid="{CD2E35A6-F544-4B63-A636-74D77758C266}"/>
+    <hyperlink ref="F4" r:id="rId18" xr:uid="{F3943AA0-1471-4D0C-BBB5-13FA0FC276C0}"/>
+    <hyperlink ref="D4" r:id="rId19" xr:uid="{1EFEDA74-BF37-4EFE-ADF1-10A85C773490}"/>
+    <hyperlink ref="F7" r:id="rId20" xr:uid="{D1B9C0A9-C86C-4C80-89C5-7E8FB7329756}"/>
+    <hyperlink ref="D7" r:id="rId21" xr:uid="{AB09AABC-8542-4C1B-B8C5-72F1265B0E68}"/>
+    <hyperlink ref="D12" r:id="rId22" xr:uid="{62176705-D2FC-4268-ABD3-057A35FD362A}"/>
+    <hyperlink ref="F12" r:id="rId23" xr:uid="{A2C833B1-ED48-4C7A-90BF-A2FC3DB7DD7F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>